<commit_message>
Update tabela de extração download file
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/tabela-extracao.xlsx
+++ b/assets/tabela-extracao.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrosandes/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CB6A47E-4882-784D-A0F5-98CBA77B98FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D2D3BB-DA6B-E840-A445-916D620EF79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19540" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Author, year</t>
   </si>
@@ -30,36 +30,6 @@
   </si>
   <si>
     <t>Groups</t>
-  </si>
-  <si>
-    <t>Brust, 1990</t>
-  </si>
-  <si>
-    <t>González, 2014</t>
-  </si>
-  <si>
-    <t>Kannoth, 2007</t>
-  </si>
-  <si>
-    <t>Lasjaunias, 2005</t>
-  </si>
-  <si>
-    <t>Matsubara, 2015</t>
-  </si>
-  <si>
-    <t>Monsuez, 1989</t>
-  </si>
-  <si>
-    <t>Nakahara, 2006</t>
-  </si>
-  <si>
-    <t>Park, 2017</t>
-  </si>
-  <si>
-    <t>Phuong, 2002</t>
-  </si>
-  <si>
-    <t>Shi, 2021</t>
   </si>
   <si>
     <t>Singla, 2015</t>
@@ -104,7 +74,40 @@
     <t>Mortality</t>
   </si>
   <si>
-    <t>Chun, 2001 </t>
+    <t>Brust 1990</t>
+  </si>
+  <si>
+    <t>Chun 2001 </t>
+  </si>
+  <si>
+    <t>González 2014</t>
+  </si>
+  <si>
+    <t>Kannoth 2007</t>
+  </si>
+  <si>
+    <t>Lasjaunias 2005</t>
+  </si>
+  <si>
+    <t>Matsubara 2015</t>
+  </si>
+  <si>
+    <t>Monsuez 1989</t>
+  </si>
+  <si>
+    <t>Nakahara 2006</t>
+  </si>
+  <si>
+    <t>Park 2017</t>
+  </si>
+  <si>
+    <t>Phuong 2002</t>
+  </si>
+  <si>
+    <t>Shi 2021</t>
+  </si>
+  <si>
+    <t>Singla 2015</t>
   </si>
 </sst>
 </file>
@@ -230,13 +233,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -245,13 +242,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -491,28 +494,28 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
@@ -534,21 +537,21 @@
       <c r="AB1" s="4"/>
     </row>
     <row r="2" spans="1:28" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="6" t="s">
-        <v>13</v>
+      <c r="A2" s="13" t="s">
+        <v>3</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
@@ -566,19 +569,19 @@
       <c r="AB2" s="4"/>
     </row>
     <row r="3" spans="1:28" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
@@ -30147,12 +30150,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A2:A3"/>
     <mergeCell ref="K2:K3"/>
     <mergeCell ref="L2:L3"/>
     <mergeCell ref="M2:M3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
-    <mergeCell ref="A2:A3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -30167,244 +30170,244 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="11"/>
+    </row>
+    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="9">
+        <v>2</v>
+      </c>
+      <c r="C2" s="9">
+        <v>13</v>
+      </c>
+      <c r="D2" s="9">
+        <v>2</v>
+      </c>
+      <c r="E2" s="9">
+        <v>5</v>
+      </c>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+    </row>
+    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="9">
+        <v>1</v>
+      </c>
+      <c r="C3" s="9">
+        <v>15</v>
+      </c>
+      <c r="D3" s="9">
+        <v>1</v>
+      </c>
+      <c r="E3" s="9">
+        <v>5</v>
+      </c>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+    </row>
+    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="9">
+        <v>0</v>
+      </c>
+      <c r="C4" s="9">
+        <v>6</v>
+      </c>
+      <c r="D4" s="9">
+        <v>3</v>
+      </c>
+      <c r="E4" s="9">
+        <v>6</v>
+      </c>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+    </row>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="9">
+        <v>1</v>
+      </c>
+      <c r="C5" s="9">
+        <v>11</v>
+      </c>
+      <c r="D5" s="9">
+        <v>3</v>
+      </c>
+      <c r="E5" s="9">
+        <v>10</v>
+      </c>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+    </row>
+    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B6" s="9">
+        <v>0</v>
+      </c>
+      <c r="C6" s="9">
+        <v>1</v>
+      </c>
+      <c r="D6" s="9">
+        <v>2</v>
+      </c>
+      <c r="E6" s="9">
+        <v>6</v>
+      </c>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+    </row>
+    <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="B7" s="9">
+        <v>2</v>
+      </c>
+      <c r="C7" s="9">
+        <v>16</v>
+      </c>
+      <c r="D7" s="9">
+        <v>0</v>
+      </c>
+      <c r="E7" s="9">
+        <v>7</v>
+      </c>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+    </row>
+    <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="B8" s="9">
+        <v>1</v>
+      </c>
+      <c r="C8" s="9">
+        <v>6</v>
+      </c>
+      <c r="D8" s="9">
+        <v>0</v>
+      </c>
+      <c r="E8" s="9">
+        <v>4</v>
+      </c>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+    </row>
+    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A9" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="B9" s="9">
+        <v>0</v>
+      </c>
+      <c r="C9" s="9">
+        <v>3</v>
+      </c>
+      <c r="D9" s="9">
+        <v>0</v>
+      </c>
+      <c r="E9" s="9">
+        <v>1</v>
+      </c>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+    </row>
+    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="B10" s="9">
+        <v>0</v>
+      </c>
+      <c r="C10" s="9">
+        <v>4</v>
+      </c>
+      <c r="D10" s="9">
+        <v>0</v>
+      </c>
+      <c r="E10" s="9">
+        <v>21</v>
+      </c>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+    </row>
+    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A11" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="G1" s="13"/>
-    </row>
-    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="11" t="s">
+      <c r="B11" s="9">
+        <v>0</v>
+      </c>
+      <c r="C11" s="9">
+        <v>10</v>
+      </c>
+      <c r="D11" s="9">
+        <v>2</v>
+      </c>
+      <c r="E11" s="9">
+        <v>5</v>
+      </c>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+    </row>
+    <row r="12" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="9">
         <v>3</v>
       </c>
-      <c r="B2" s="11">
-        <v>2</v>
+      <c r="C12" s="9">
+        <v>16</v>
       </c>
-      <c r="C2" s="11">
-        <v>13</v>
-      </c>
-      <c r="D2" s="11">
-        <v>2</v>
-      </c>
-      <c r="E2" s="11">
-        <v>5</v>
-      </c>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-    </row>
-    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="11">
-        <v>1</v>
-      </c>
-      <c r="C3" s="11">
-        <v>15</v>
-      </c>
-      <c r="D3" s="11">
-        <v>1</v>
-      </c>
-      <c r="E3" s="11">
-        <v>5</v>
-      </c>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-    </row>
-    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="11">
-        <v>0</v>
-      </c>
-      <c r="C4" s="11">
-        <v>6</v>
-      </c>
-      <c r="D4" s="11">
+      <c r="D12" s="9">
         <v>3</v>
       </c>
-      <c r="E4" s="11">
-        <v>6</v>
-      </c>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-    </row>
-    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="11">
-        <v>1</v>
-      </c>
-      <c r="C5" s="11">
-        <v>11</v>
-      </c>
-      <c r="D5" s="11">
-        <v>3</v>
-      </c>
-      <c r="E5" s="11">
-        <v>10</v>
-      </c>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-    </row>
-    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="11">
-        <v>0</v>
-      </c>
-      <c r="C6" s="11">
-        <v>1</v>
-      </c>
-      <c r="D6" s="11">
-        <v>2</v>
-      </c>
-      <c r="E6" s="11">
-        <v>6</v>
-      </c>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-    </row>
-    <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A7" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="11">
-        <v>2</v>
-      </c>
-      <c r="C7" s="11">
-        <v>16</v>
-      </c>
-      <c r="D7" s="11">
-        <v>0</v>
-      </c>
-      <c r="E7" s="11">
-        <v>7</v>
-      </c>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-    </row>
-    <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="11">
-        <v>1</v>
-      </c>
-      <c r="C8" s="11">
-        <v>6</v>
-      </c>
-      <c r="D8" s="11">
-        <v>0</v>
-      </c>
-      <c r="E8" s="11">
-        <v>4</v>
-      </c>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-    </row>
-    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="11">
-        <v>0</v>
-      </c>
-      <c r="C9" s="11">
-        <v>3</v>
-      </c>
-      <c r="D9" s="11">
-        <v>0</v>
-      </c>
-      <c r="E9" s="11">
-        <v>1</v>
-      </c>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-    </row>
-    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="11">
-        <v>0</v>
-      </c>
-      <c r="C10" s="11">
-        <v>4</v>
-      </c>
-      <c r="D10" s="11">
-        <v>0</v>
-      </c>
-      <c r="E10" s="11">
-        <v>21</v>
-      </c>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-    </row>
-    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A11" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="11">
-        <v>0</v>
-      </c>
-      <c r="C11" s="11">
-        <v>10</v>
-      </c>
-      <c r="D11" s="11">
-        <v>2</v>
-      </c>
-      <c r="E11" s="11">
-        <v>5</v>
-      </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-    </row>
-    <row r="12" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A12" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="11">
-        <v>3</v>
-      </c>
-      <c r="C12" s="11">
-        <v>16</v>
-      </c>
-      <c r="D12" s="11">
-        <v>3</v>
-      </c>
-      <c r="E12" s="11">
+      <c r="E12" s="9">
         <v>19</v>
       </c>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
     </row>
     <row r="13" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
-        <v>13</v>
+      <c r="A13" s="12" t="s">
+        <v>28</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="13"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>